<commit_message>
Release SMD CVMod8 V2.
</commit_message>
<xml_diff>
--- a/Modules/CVMod8_V2/CVMod8_V2_BOM.xlsx
+++ b/Modules/CVMod8_V2/CVMod8_V2_BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\My-Dev\Modular Synth\Avalon Harmonics\CVMod8_V2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DB19257-EAEE-482B-A79F-2FB7D0BA5639}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{077031D6-058E-4C5F-9902-ACF7108DD09D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="109">
   <si>
     <t>Qty</t>
   </si>
@@ -56,9 +56,6 @@
     <t>47uF</t>
   </si>
   <si>
-    <t>1N4001</t>
-  </si>
-  <si>
     <t>D1, D2</t>
   </si>
   <si>
@@ -74,18 +71,6 @@
     <t>TL074</t>
   </si>
   <si>
-    <t>R-Array-SIP8</t>
-  </si>
-  <si>
-    <t>Resistor THT</t>
-  </si>
-  <si>
-    <t>DIP-14</t>
-  </si>
-  <si>
-    <t>Quad Op Amp</t>
-  </si>
-  <si>
     <t>PWR</t>
   </si>
   <si>
@@ -104,18 +89,6 @@
     <t>Slide Potentiometer</t>
   </si>
   <si>
-    <t>Rectifier Diode</t>
-  </si>
-  <si>
-    <t>DO-41</t>
-  </si>
-  <si>
-    <t>IC Socket</t>
-  </si>
-  <si>
-    <t>DIP-14 Socket</t>
-  </si>
-  <si>
     <t>Link</t>
   </si>
   <si>
@@ -128,18 +101,6 @@
     <t>https://www.thonk.co.uk/shop/ttpots/</t>
   </si>
   <si>
-    <t>https://www.aliexpress.com/item/1005002670881002.html</t>
-  </si>
-  <si>
-    <t>https://www.aliexpress.com/item/1005003256812123.html</t>
-  </si>
-  <si>
-    <t>Male Header 2.54mm</t>
-  </si>
-  <si>
-    <t>1x3</t>
-  </si>
-  <si>
     <t>2x5</t>
   </si>
   <si>
@@ -185,9 +146,6 @@
     <t>Potentiometer Plastic</t>
   </si>
   <si>
-    <t>https://www.aliexpress.com/item/1005003256254825.html</t>
-  </si>
-  <si>
     <t>C1, C2</t>
   </si>
   <si>
@@ -209,24 +167,9 @@
     <t>B100k PTA3043 -2015DPB104</t>
   </si>
   <si>
-    <t>1x6</t>
-  </si>
-  <si>
-    <t>Female Header 2.54mm</t>
-  </si>
-  <si>
     <t>78L05</t>
   </si>
   <si>
-    <t>TO-92 Wide</t>
-  </si>
-  <si>
-    <t>Voltage Regulator 5V</t>
-  </si>
-  <si>
-    <t>Voltage Regulator -5V NEGATIVE</t>
-  </si>
-  <si>
     <t>79L05</t>
   </si>
   <si>
@@ -245,9 +188,6 @@
     <t>https://www.thonk.co.uk/shop/sub-mini-toggle-switches/</t>
   </si>
   <si>
-    <t>U1 - U8</t>
-  </si>
-  <si>
     <t>M2*5</t>
   </si>
   <si>
@@ -266,18 +206,9 @@
     <t>https://www.aliexpress.com/item/1005002177898963.html</t>
   </si>
   <si>
-    <t>M2, 11mm</t>
-  </si>
-  <si>
-    <t>M2 Standoff</t>
-  </si>
-  <si>
     <t>Standoff</t>
   </si>
   <si>
-    <t>https://www.aliexpress.com/item/1005002952338852.html</t>
-  </si>
-  <si>
     <r>
       <t>Bourns Slide Pot 30mm, 15mm L</t>
     </r>
@@ -317,6 +248,414 @@
     </r>
   </si>
   <si>
+    <t>*** For SW_FWD switches, don't use the nut between the panel and the switch. These switches should not be pressed against the PCB, but "hover" instead. The legs will be a bit shorter when poking through the PCB holes, but should still be solderable.</t>
+  </si>
+  <si>
+    <r>
+      <t>Sub-Mini SPDT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>***</t>
+    </r>
+  </si>
+  <si>
+    <t>Thonkiconn</t>
+  </si>
+  <si>
+    <t>Alt Link</t>
+  </si>
+  <si>
+    <t>https://www.mouser.de/ProductDetail/Bourns/PTA3043-2015DPB104?qs=zRGnDeWDVj0fVt3rAxibYA%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/de/en/details/l-937egw/tht-leds-3mm/kingbright-electronic/</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/de/en/details/zl202-80g/pin-headers/connfly/ds1021-2-40sf11/</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/de/en/details/tfm-m2x10_dr211of/metal-spacers/dremec/211x10of/</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>P_ATN1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>P_ATN8</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>P_OFS1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>P_OFS8</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>LD1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>LD8</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SW_POL1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SW_POL8</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SW_FWD1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SW_FWD7</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>J_IN1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>J_IN8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> J_OUT1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>J_OUT8</t>
+    </r>
+  </si>
+  <si>
+    <t>C3-C14</t>
+  </si>
+  <si>
+    <t>LED 3mm Dome Bicolor</t>
+  </si>
+  <si>
+    <t>R-0603</t>
+  </si>
+  <si>
+    <t>Parts  with underline are on the front side of the PCB!</t>
+  </si>
+  <si>
+    <t>R1-R16</t>
+  </si>
+  <si>
+    <t>R17-R79</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/de/en/details/smd0603-1k-1%25/smd-resistors/royalohm/0603saf1001t5e/</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/de/en/details/smd0603-100k-1%25/smd-resistors/royalohm/0603saf1003t5e/</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/de/en/details/0603b104k500ct/mlcc-smd-capacitors/walsin/</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/de/en/details/sc1e476m6l005vr/smd-electrolytic-capacitors/samwha/</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/de/en/details/fm4001-lge/smd-universal-diodes/luguang-electronic/fm4001/</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/de/en/details/tl074bcdt/smd-operational-amplifiers/stmicroelectronics/</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/de/en/details/l78l05abutr/fixed-voltage-regulators/stmicroelectronics/</t>
+  </si>
+  <si>
+    <t>https://www.tme.eu/de/en/details/lm79l05a-cdi/fixed-voltage-regulators/cdil/lm79l05a/</t>
+  </si>
+  <si>
+    <t>Resistor SMD</t>
+  </si>
+  <si>
+    <t>Ceramic Capacitor SMD</t>
+  </si>
+  <si>
+    <t>Electrolytic Capacitor SMD</t>
+  </si>
+  <si>
+    <t>Rectifier Diode SMD</t>
+  </si>
+  <si>
+    <t>Quad Op Amp SMD</t>
+  </si>
+  <si>
+    <t>Voltage Regulator 5V SMD</t>
+  </si>
+  <si>
+    <t>Voltage Regulator -5V NEGATIVE SMD</t>
+  </si>
+  <si>
+    <t>C-0603</t>
+  </si>
+  <si>
+    <t>E-6.3x5.3mm</t>
+  </si>
+  <si>
+    <t>FM4001</t>
+  </si>
+  <si>
+    <t>SOD123F</t>
+  </si>
+  <si>
+    <t>SO14</t>
+  </si>
+  <si>
+    <t>U1-U8</t>
+  </si>
+  <si>
+    <t>SOT89</t>
+  </si>
+  <si>
+    <t>**** Snip off the pins below the switch almost flush to the PCB, otherwise you won't be able to mount the switch.</t>
+  </si>
+  <si>
+    <t>***** 10mm standoffs are used between the panel and main PCB. Orient them so that the screws go in from the panel side.</t>
+  </si>
+  <si>
+    <t>****** Don't push the caps all the way down, otherwise they will slightly scrape against the panel.</t>
+  </si>
+  <si>
+    <r>
+      <t>Male Header 2.54mm</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>****</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>M2 Standoff</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>*****</t>
+    </r>
+  </si>
+  <si>
     <r>
       <t>Sifam Sleek Slider Cap</t>
     </r>
@@ -328,506 +667,11 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>*****</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>M2 Standoff</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>****</t>
-    </r>
-  </si>
-  <si>
-    <t>**** 10mm standoffs are used between the panel and front PCB, while the 11mm ones are used between the main PCB and front PCB. For the 10mm ones, orient them so that the screws go in from the panel side.</t>
-  </si>
-  <si>
-    <t>***** Don't push the caps all the way down, otherwise they will slightly scrape against the panel.</t>
-  </si>
-  <si>
-    <t>*** For SW_FWD switches, don't use the nut between the panel and the switch. These switches should not be pressed against the PCB, but "hover" instead. The legs will be a bit shorter when poking through the PCB holes, but should still be solderable.</t>
-  </si>
-  <si>
-    <r>
-      <t>Sub-Mini SPDT</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>***</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Resistor Network THT, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>4 Isolated Resistors</t>
-    </r>
-  </si>
-  <si>
-    <t>Thonkiconn</t>
-  </si>
-  <si>
-    <t>R-1/4W</t>
-  </si>
-  <si>
-    <t>C-P5mm</t>
-  </si>
-  <si>
-    <t>E-P2.5mm 6.3x11.5mm</t>
-  </si>
-  <si>
-    <t>Electrolytic Capacitor THT</t>
-  </si>
-  <si>
-    <t>Ceramic Capacitor THT</t>
-  </si>
-  <si>
-    <t>Alt Link</t>
-  </si>
-  <si>
-    <t>https://www.mouser.de/ProductDetail/Bourns/PTA3043-2015DPB104?qs=zRGnDeWDVj0fVt3rAxibYA%3D%3D</t>
-  </si>
-  <si>
-    <t>https://www.buerklin.com/en/p/quadrios/wirewound-resistors/22p046/73P0034/</t>
-  </si>
-  <si>
-    <t>https://www.tme.eu/de/en/details/icvt-14p/standard-dip-sockets/connfly/ds1009-14at1nx-0a2/</t>
-  </si>
-  <si>
-    <t>https://www.tme.eu/de/en/details/zl262-3sg/pin-headers/connfly/ds1023-1-3s21/</t>
-  </si>
-  <si>
-    <t>https://www.tme.eu/de/en/details/zl262-6sg/pin-headers/connfly/ds1023-1-6s21/</t>
+      <t>******</t>
+    </r>
   </si>
   <si>
     <t>Avalon Harmonics CVMod8 V2</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>Parts  with underline are on the front PCB!</t>
-  </si>
-  <si>
-    <t>https://www.tme.eu/de/en/details/dr100k-4_8/resistor-networks/royal-ohm/rnlb08g0104b0e/</t>
-  </si>
-  <si>
-    <t>https://www.tme.eu/de/en/details/cm-100n-x7r_100/mlcc-tht-capacitors/sr-passives/</t>
-  </si>
-  <si>
-    <t>https://www.tme.eu/de/en/details/jrg-47u_35/tht-electrolytic-capacitors/jb-capacitors/jrg1v470m02500630115000b/</t>
-  </si>
-  <si>
-    <t>https://www.tme.eu/de/en/details/1n4001-dio/tht-universal-diodes/diotec-semiconductor/1n4001/</t>
-  </si>
-  <si>
-    <t>https://www.tme.eu/de/en/details/tl074acn/tht-operational-amplifiers/texas-instruments/</t>
-  </si>
-  <si>
-    <t>https://www.tme.eu/de/en/details/l78l05abz/unregulated-voltage-regulators/stmicroelectronics/</t>
-  </si>
-  <si>
-    <t>https://www.tme.eu/de/en/details/l79l05acz/unregulated-voltage-regulators/stmicroelectronics/</t>
-  </si>
-  <si>
-    <t>https://www.tme.eu/de/en/details/l-937egw/tht-leds-3mm/kingbright-electronic/</t>
-  </si>
-  <si>
-    <t>https://www.tme.eu/de/en/details/zl201-40g/pin-headers/connfly/ds1021-1-40sf11-b/</t>
-  </si>
-  <si>
-    <t>https://www.tme.eu/de/en/details/zl202-80g/pin-headers/connfly/ds1021-2-40sf11/</t>
-  </si>
-  <si>
-    <t>https://www.tme.eu/de/en/details/tfm-m2x10_dr211of/metal-spacers/dremec/211x10of/</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>P_ATN1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>-</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>P_ATN8</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>P_OFS1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>-</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>P_OFS8</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>LD1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>-</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>LD8</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SW_POL1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>-</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SW_POL8</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SW_FWD1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>-</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SW_FWD7</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>J_IN1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>-</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>J_IN8</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>,</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> J_OUT1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>-</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>J_OUT8</t>
-    </r>
-  </si>
-  <si>
-    <t>J_A1-J_A8</t>
-  </si>
-  <si>
-    <t>J_A11-J_A14</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>J_B1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>-</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>J_B8</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>J_B11</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>-</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>J_B14</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">R1-R8, </t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>R11</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>-</t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>R18</t>
-    </r>
-  </si>
-  <si>
-    <t>RN1-RN16</t>
-  </si>
-  <si>
-    <t>C3-C14</t>
-  </si>
-  <si>
-    <t>LED 3mm Dome Bicolor</t>
   </si>
 </sst>
 </file>
@@ -1718,20 +1562,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.7109375" customWidth="1"/>
     <col min="2" max="2" width="28.42578125" customWidth="1"/>
     <col min="3" max="3" width="34.85546875" customWidth="1"/>
     <col min="4" max="4" width="27.5703125" customWidth="1"/>
-    <col min="5" max="5" width="38.85546875" customWidth="1"/>
+    <col min="5" max="5" width="36.42578125" customWidth="1"/>
     <col min="6" max="6" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -1751,11 +1595,11 @@
         <v>4</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="G2" s="1"/>
       <c r="J2" s="1" t="s">
-        <v>95</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -1763,45 +1607,45 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="D3" t="s">
-        <v>125</v>
+        <v>78</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>88</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>97</v>
+        <v>80</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>31</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>16</v>
+        <v>63</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>76</v>
       </c>
       <c r="D4" t="s">
-        <v>126</v>
+        <v>79</v>
       </c>
       <c r="E4" t="s">
         <v>88</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>50</v>
+        <v>81</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>104</v>
+        <v>64</v>
       </c>
       <c r="L4" s="3"/>
     </row>
@@ -1813,19 +1657,19 @@
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D5" t="s">
-        <v>127</v>
+        <v>74</v>
       </c>
       <c r="E5" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>105</v>
+        <v>82</v>
       </c>
       <c r="J5" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -1836,19 +1680,19 @@
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D6" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="E6" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>106</v>
+        <v>83</v>
       </c>
       <c r="J6" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -1856,22 +1700,22 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D7" t="s">
         <v>7</v>
       </c>
-      <c r="C7" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" t="s">
-        <v>8</v>
-      </c>
       <c r="E7" t="s">
-        <v>23</v>
+        <v>91</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="J7" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -1879,45 +1723,45 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>99</v>
       </c>
       <c r="D8" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="E8" t="s">
-        <v>25</v>
+        <v>92</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>32</v>
+        <v>85</v>
+      </c>
+      <c r="J8" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>101</v>
       </c>
       <c r="D9" t="s">
-        <v>66</v>
+        <v>42</v>
       </c>
       <c r="E9" t="s">
-        <v>16</v>
+        <v>93</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="J9" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -1925,45 +1769,42 @@
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="C10" t="s">
-        <v>57</v>
+        <v>101</v>
       </c>
       <c r="D10" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="E10" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>109</v>
+        <v>87</v>
       </c>
       <c r="J10" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>60</v>
+        <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="E11" t="s">
-        <v>59</v>
+        <v>36</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="J11" t="s">
-        <v>102</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -1971,19 +1812,22 @@
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D12" t="s">
-        <v>115</v>
+        <v>69</v>
       </c>
       <c r="E12" t="s">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>30</v>
+        <v>63</v>
+      </c>
+      <c r="J12" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
@@ -1991,22 +1835,22 @@
         <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>53</v>
+        <v>16</v>
       </c>
       <c r="C13" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D13" t="s">
-        <v>116</v>
+        <v>70</v>
       </c>
       <c r="E13" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="J13" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -2014,114 +1858,91 @@
         <v>8</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="C14" t="s">
-        <v>128</v>
+        <v>58</v>
       </c>
       <c r="D14" t="s">
-        <v>117</v>
+        <v>71</v>
       </c>
       <c r="E14" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>111</v>
+        <v>46</v>
       </c>
       <c r="J14" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B15" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="C15" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="D15" t="s">
-        <v>118</v>
+        <v>72</v>
       </c>
       <c r="E15" t="s">
+        <v>45</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="J15" t="s">
         <v>64</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="J15" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C16" t="s">
-        <v>87</v>
+        <v>19</v>
       </c>
       <c r="D16" t="s">
-        <v>119</v>
+        <v>73</v>
       </c>
       <c r="E16" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J16" t="s">
         <v>64</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="J16" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="B17" t="s">
-        <v>89</v>
+        <v>22</v>
       </c>
       <c r="C17" t="s">
-        <v>28</v>
+        <v>105</v>
       </c>
       <c r="D17" t="s">
-        <v>120</v>
+        <v>12</v>
       </c>
       <c r="E17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>29</v>
+        <v>66</v>
       </c>
       <c r="J17" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>8</v>
-      </c>
-      <c r="B18" t="s">
-        <v>54</v>
-      </c>
-      <c r="C18" t="s">
-        <v>33</v>
-      </c>
-      <c r="D18" t="s">
-        <v>121</v>
-      </c>
-      <c r="E18" t="s">
-        <v>19</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="J18" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -2129,45 +1950,39 @@
         <v>4</v>
       </c>
       <c r="B19" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="C19" t="s">
         <v>33</v>
       </c>
-      <c r="D19" t="s">
-        <v>122</v>
-      </c>
       <c r="E19" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>112</v>
+        <v>34</v>
       </c>
       <c r="J19" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B20" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C20" t="s">
-        <v>55</v>
-      </c>
-      <c r="D20" t="s">
-        <v>123</v>
+        <v>50</v>
       </c>
       <c r="E20" t="s">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="J20" s="3" t="s">
-        <v>102</v>
+        <v>52</v>
+      </c>
+      <c r="J20" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -2175,45 +1990,42 @@
         <v>4</v>
       </c>
       <c r="B21" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="C21" t="s">
-        <v>55</v>
-      </c>
-      <c r="D21" t="s">
-        <v>124</v>
+        <v>106</v>
       </c>
       <c r="E21" t="s">
-        <v>19</v>
+        <v>53</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="J21" s="3" t="s">
-        <v>102</v>
+        <v>67</v>
+      </c>
+      <c r="J21" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>1</v>
-      </c>
-      <c r="B22" t="s">
+      <c r="F22" s="3"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>8</v>
+      </c>
+      <c r="B23" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" t="s">
+        <v>29</v>
+      </c>
+      <c r="E23" t="s">
         <v>35</v>
       </c>
-      <c r="C22" t="s">
-        <v>33</v>
-      </c>
-      <c r="D22" t="s">
-        <v>17</v>
-      </c>
-      <c r="E22" t="s">
-        <v>19</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="J22" t="s">
-        <v>102</v>
+      <c r="F23" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="J23" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
@@ -2221,19 +2033,19 @@
         <v>8</v>
       </c>
       <c r="B24" t="s">
-        <v>67</v>
+        <v>31</v>
       </c>
       <c r="C24" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="E24" t="s">
-        <v>68</v>
+        <v>35</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="J24" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
@@ -2241,223 +2053,114 @@
         <v>8</v>
       </c>
       <c r="B25" t="s">
-        <v>69</v>
+        <v>24</v>
       </c>
       <c r="C25" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="E25" t="s">
-        <v>71</v>
+        <v>27</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="J25" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B26" t="s">
-        <v>78</v>
+        <v>24</v>
       </c>
       <c r="C26" t="s">
-        <v>83</v>
+        <v>107</v>
       </c>
       <c r="E26" t="s">
-        <v>75</v>
+        <v>26</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>114</v>
+        <v>28</v>
       </c>
       <c r="J26" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B28" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B29" s="2"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B30" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B31" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B32" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B33" s="4" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>4</v>
-      </c>
-      <c r="B27" t="s">
-        <v>73</v>
-      </c>
-      <c r="C27" t="s">
-        <v>74</v>
-      </c>
-      <c r="E27" t="s">
-        <v>75</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="J27" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F28" s="3"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29">
-        <v>8</v>
-      </c>
-      <c r="B29" t="s">
-        <v>37</v>
-      </c>
-      <c r="C29" t="s">
-        <v>42</v>
-      </c>
-      <c r="E29" t="s">
-        <v>48</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="J29" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30">
-        <v>8</v>
-      </c>
-      <c r="B30" t="s">
-        <v>44</v>
-      </c>
-      <c r="C30" t="s">
-        <v>42</v>
-      </c>
-      <c r="E30" t="s">
-        <v>48</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="J30" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31">
-        <v>8</v>
-      </c>
-      <c r="B31" t="s">
-        <v>37</v>
-      </c>
-      <c r="C31" t="s">
-        <v>36</v>
-      </c>
-      <c r="E31" t="s">
-        <v>40</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="J31" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <v>8</v>
-      </c>
-      <c r="B32" t="s">
-        <v>37</v>
-      </c>
-      <c r="C32" t="s">
-        <v>82</v>
-      </c>
-      <c r="E32" t="s">
-        <v>39</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="J32" t="s">
-        <v>102</v>
-      </c>
-    </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="4" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B35" s="2"/>
+      <c r="B35" s="4" t="s">
+        <v>104</v>
+      </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B36" s="4" t="s">
-        <v>79</v>
-      </c>
+      <c r="A36" s="1"/>
+      <c r="F36" s="3"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B37" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B38" s="4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B39" s="4" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B40" s="4" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42" s="1"/>
-      <c r="F42" s="3"/>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C43" s="3"/>
-      <c r="G43" s="1"/>
-      <c r="J43" s="3"/>
+      <c r="C37" s="3"/>
+      <c r="G37" s="1"/>
+      <c r="J37" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F14" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="F17" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="F12" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="F9" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="F7" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="F6" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="F5" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="J4" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="J8" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="J3" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="F31" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="F29" r:id="rId12" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="F30" r:id="rId13" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="F32" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="J20" r:id="rId15" display="https://www.aliexpress.com/item/1005001557138121.html" xr:uid="{87917B98-45C2-4356-99DB-B5B8038C28A9}"/>
-    <hyperlink ref="F18" r:id="rId16" xr:uid="{7E9B1C1C-08C2-4E3A-836F-A55BD1AACB08}"/>
-    <hyperlink ref="J21" r:id="rId17" display="https://www.aliexpress.com/item/1005001557138121.html" xr:uid="{3932249F-F50C-48B7-B9ED-979BED78C705}"/>
-    <hyperlink ref="F19" r:id="rId18" xr:uid="{617026E1-E8F8-41F0-B6F6-C7F3EABF9EDE}"/>
-    <hyperlink ref="F10" r:id="rId19" xr:uid="{D97E84B0-51EF-4445-A800-1CCE20EEB5DD}"/>
-    <hyperlink ref="F11" r:id="rId20" xr:uid="{37603052-44CC-44A4-A373-590BE7540B20}"/>
-    <hyperlink ref="F16" r:id="rId21" xr:uid="{57A67E62-1F07-4F81-BD71-0FCCC53DDD36}"/>
-    <hyperlink ref="F24" r:id="rId22" xr:uid="{386CA78F-ECAF-4BED-B017-86D6F4F05D83}"/>
-    <hyperlink ref="F25" r:id="rId23" xr:uid="{23053745-F5D1-4E91-88AD-FDB570AEC8C5}"/>
-    <hyperlink ref="F27" r:id="rId24" xr:uid="{3EC41E3D-44DB-45CF-A556-8137102A88B8}"/>
-    <hyperlink ref="F15" r:id="rId25" xr:uid="{11ED5ED0-56A5-4C20-93A1-FDAE72827046}"/>
-    <hyperlink ref="F22" r:id="rId26" xr:uid="{A893ABC8-5223-47F2-8335-C8AD6F9E7D68}"/>
-    <hyperlink ref="F4" r:id="rId27" xr:uid="{D1B00FCF-CFA9-4559-AFDD-E930832032EF}"/>
-    <hyperlink ref="F13" r:id="rId28" xr:uid="{29AEA817-32F1-41F4-A924-4F4000D4818B}"/>
-    <hyperlink ref="F3" r:id="rId29" xr:uid="{8A7A5D82-A3F8-44CA-BA5B-9240FAD7EA78}"/>
-    <hyperlink ref="F8" r:id="rId30" xr:uid="{5987D41B-D98C-45BC-A0CC-34272D97726E}"/>
-    <hyperlink ref="F21" r:id="rId31" xr:uid="{8E872B71-2423-4E3E-A4A8-BAD79ACAED0B}"/>
-    <hyperlink ref="F20" r:id="rId32" xr:uid="{7AFABD24-8F23-415C-8FB0-53C856BB2EE7}"/>
-    <hyperlink ref="F26" r:id="rId33" xr:uid="{43A1E3D1-40BA-485C-A829-B483D6181C61}"/>
+    <hyperlink ref="F13" r:id="rId1" xr:uid="{13764AEB-15A6-4D90-ABE7-2699FFC21667}"/>
+    <hyperlink ref="F16" r:id="rId2" xr:uid="{132D58BF-3722-4009-997D-85D83E0427E1}"/>
+    <hyperlink ref="F11" r:id="rId3" xr:uid="{8566253D-4BC4-4E88-AEC8-42702836E845}"/>
+    <hyperlink ref="F25" r:id="rId4" xr:uid="{F21785D4-9E60-49FA-B073-FBF9DF240B91}"/>
+    <hyperlink ref="F23" r:id="rId5" xr:uid="{95AE4A90-92CF-45E8-81B2-053915D45020}"/>
+    <hyperlink ref="F24" r:id="rId6" xr:uid="{21D8AB96-92BC-4134-9A7C-8F0559A3B677}"/>
+    <hyperlink ref="F26" r:id="rId7" xr:uid="{01A30E79-E5B2-47BA-A3E7-2780BB7C6150}"/>
+    <hyperlink ref="F15" r:id="rId8" xr:uid="{6A2C0C52-D1AE-4FD1-A752-B35B8C35F326}"/>
+    <hyperlink ref="F19" r:id="rId9" xr:uid="{4950D606-84F3-4140-9E5E-B30237872926}"/>
+    <hyperlink ref="F20" r:id="rId10" xr:uid="{598DC950-F0D5-4E2E-8295-A9654732F752}"/>
+    <hyperlink ref="F14" r:id="rId11" xr:uid="{85CF4EAD-C815-4764-99B0-3CD3F7C65648}"/>
+    <hyperlink ref="F17" r:id="rId12" xr:uid="{E5E643F1-584B-4524-8FC0-A33A6B86DA13}"/>
+    <hyperlink ref="F12" r:id="rId13" xr:uid="{F9D4FE49-B4B1-48B5-AA25-31D2A78EB9EB}"/>
+    <hyperlink ref="F21" r:id="rId14" xr:uid="{C4F7CA67-414F-44EB-8D12-BDA7608A9909}"/>
+    <hyperlink ref="F7" r:id="rId15" xr:uid="{50D31F83-0CC7-4366-B19A-AB742DEC9C95}"/>
+    <hyperlink ref="F8" r:id="rId16" xr:uid="{8A08C8AB-0BC2-48C9-839C-9A1FF04B94D0}"/>
+    <hyperlink ref="F6" r:id="rId17" xr:uid="{8CB4637D-11ED-44D2-995C-63FD7A7880CC}"/>
+    <hyperlink ref="F5" r:id="rId18" xr:uid="{950D2F1D-A663-4192-B413-DEF807105565}"/>
+    <hyperlink ref="F3" r:id="rId19" xr:uid="{148C00D5-077D-40A7-90B4-A86DC721AC43}"/>
+    <hyperlink ref="F9" r:id="rId20" xr:uid="{4B8DCC33-CC14-4260-9B2A-502EFE5C16D7}"/>
+    <hyperlink ref="F10" r:id="rId21" xr:uid="{0985F146-BC4A-4DC8-A796-B9EBFBBF916A}"/>
+    <hyperlink ref="F4" r:id="rId22" xr:uid="{39108D5A-B9E3-49BD-8858-806D8CB46293}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId34"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId23"/>
 </worksheet>
 </file>
</xml_diff>